<commit_message>
Update AutoTache persistent state
</commit_message>
<xml_diff>
--- a/cloud_state/offres_suivi.xlsx
+++ b/cloud_state/offres_suivi.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Offres" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offres" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Offres'!$A$1:$AB$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Offres'!$A$1:$AB$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB16"/>
+  <dimension ref="A1:AB17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -460,7 +460,7 @@
     <col width="21" customWidth="1" min="15" max="15"/>
     <col width="19" customWidth="1" min="16" max="16"/>
     <col width="57" customWidth="1" min="17" max="17"/>
-    <col width="29" customWidth="1" min="18" max="18"/>
+    <col width="35" customWidth="1" min="18" max="18"/>
     <col width="26" customWidth="1" min="19" max="19"/>
     <col width="13" customWidth="1" min="20" max="20"/>
     <col width="60" customWidth="1" min="21" max="21"/>
@@ -2150,8 +2150,104 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21T11:40:47</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>-8074488563249637161</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Développeur php full stack - h/f</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Altagile</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Sennecey-lès-Dijon, 21800</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Temps plein</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr"/>
+      <c r="N17" s="2" t="inlineStr"/>
+      <c r="O17" s="2" t="inlineStr"/>
+      <c r="P17" s="2" t="inlineStr"/>
+      <c r="Q17" s="2" t="inlineStr">
+        <is>
+          <t>JavaScript, React</t>
+        </is>
+      </c>
+      <c r="R17" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21T09:05:14.6248696+00:00</t>
+        </is>
+      </c>
+      <c r="S17" s="2" t="inlineStr"/>
+      <c r="T17" s="2" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="U17" s="2" t="inlineStr">
+        <is>
+          <t>Offre conservee: cible front-end, WordPress, webdesign, UI/UX ou graphisme web.</t>
+        </is>
+      </c>
+      <c r="V17" s="2" t="inlineStr">
+        <is>
+          <t>À vérifier</t>
+        </is>
+      </c>
+      <c r="W17" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="X17" s="2" t="inlineStr">
+        <is>
+          <t>À vérifier: score 65/100 grâce à technologies: javascript, react, web; domaine_metier: wordpress, front-end, ui, ux, design, webdesign, graphisme; localisation: dijon.</t>
+        </is>
+      </c>
+      <c r="Y17" s="2" t="inlineStr">
+        <is>
+          <t>technologies=35; titre=0; domaine_metier=15; localisation=15; teletravail=0; contrat=0</t>
+        </is>
+      </c>
+      <c r="Z17" s="2" t="inlineStr">
+        <is>
+          <t>JavaScript, React</t>
+        </is>
+      </c>
+      <c r="AA17" s="2" t="inlineStr"/>
+      <c r="AB17" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.jooble.org/jdp/-8074488563249637161</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AB16"/>
+  <autoFilter ref="A1:AB17"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB3" r:id="rId2"/>
@@ -2168,6 +2264,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB14" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB15" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB17" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>